<commit_message>
fix: improve duplicate index matching in 90 vs 99 compare export
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/internal-materials/ego-ok/items-90-vs-99-compare.xlsx
+++ b/docs/internal-materials/ego-ok/items-90-vs-99-compare.xlsx
@@ -1705,13 +1705,13 @@
         <v>ego 20</v>
       </c>
       <c r="E41">
-        <v>82</v>
+        <v>2</v>
       </c>
       <c r="F41" t="str">
         <v>a_negative</v>
       </c>
       <c r="G41" t="str">
-        <v>대체로 원칙과 효율에만 얽매여, 융통성과 인간미가 부족하다는 말을 듣곤 한다.</v>
+        <v>매사에 표정이나 감정 변화가 적어서, 사람들에게 딱딱하고 재미없다는 인상을 주는 편이다.</v>
       </c>
       <c r="H41" t="str">
         <v>Y</v>
@@ -1720,7 +1720,7 @@
         <v>N</v>
       </c>
       <c r="J41" t="str">
-        <v>인덱스 2·82번</v>
+        <v>동일인덱스 2·82 → 2번 대표</v>
       </c>
     </row>
     <row r="42">

</xml_diff>